<commit_message>
Agregar politicas y bitacora fotografica vehicular
</commit_message>
<xml_diff>
--- a/plantillas/plantilla_cuentas_docentes.xlsx
+++ b/plantillas/plantilla_cuentas_docentes.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Docentes" sheetId="1" r:id="R73e1137280c04fea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R0b4d7a9be3e645f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Docentes" sheetId="1" r:id="Ra415354427c349ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R5f211504e4634b72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="@"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -45,8 +45,14 @@
       <x:color rgb="FF65716E"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -76,6 +82,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF4F7F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F7FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF087F5B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F7FA"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -113,7 +134,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -152,6 +173,16 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -357,6 +388,7 @@
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -369,258 +401,316 @@
       <x:c r="C1" s="5" t="str">
         <x:v>Contraseña temporal</x:v>
       </x:c>
+      <x:c r="D1" s="24" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="23" customHeight="1">
       <x:c r="A2" s="9" t="str"/>
       <x:c r="B2" s="10" t="str"/>
       <x:c r="C2" s="11" t="str"/>
+      <x:c r="D2" s="25"/>
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="9" t="str"/>
       <x:c r="B3" s="10" t="str"/>
       <x:c r="C3" s="11" t="str"/>
+      <x:c r="D3" s="25"/>
     </x:row>
     <x:row r="4" ht="23" customHeight="1">
       <x:c r="A4" s="9" t="str"/>
       <x:c r="B4" s="10" t="str"/>
       <x:c r="C4" s="11" t="str"/>
+      <x:c r="D4" s="25"/>
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
       <x:c r="A5" s="9" t="str"/>
       <x:c r="B5" s="10" t="str"/>
       <x:c r="C5" s="11" t="str"/>
+      <x:c r="D5" s="25"/>
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="A6" s="9" t="str"/>
       <x:c r="B6" s="10" t="str"/>
       <x:c r="C6" s="11" t="str"/>
+      <x:c r="D6" s="25"/>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="9" t="str"/>
       <x:c r="B7" s="10" t="str"/>
       <x:c r="C7" s="11" t="str"/>
+      <x:c r="D7" s="25"/>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
       <x:c r="A8" s="9" t="str"/>
       <x:c r="B8" s="10" t="str"/>
       <x:c r="C8" s="11" t="str"/>
+      <x:c r="D8" s="25"/>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="9" t="str"/>
       <x:c r="B9" s="10" t="str"/>
       <x:c r="C9" s="11" t="str"/>
+      <x:c r="D9" s="25"/>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="9" t="str"/>
       <x:c r="B10" s="10" t="str"/>
       <x:c r="C10" s="11" t="str"/>
+      <x:c r="D10" s="25"/>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
       <x:c r="A11" s="9" t="str"/>
       <x:c r="B11" s="10" t="str"/>
       <x:c r="C11" s="11" t="str"/>
+      <x:c r="D11" s="25"/>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="9" t="str"/>
       <x:c r="B12" s="10" t="str"/>
       <x:c r="C12" s="11" t="str"/>
+      <x:c r="D12" s="25"/>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
       <x:c r="A13" s="9" t="str"/>
       <x:c r="B13" s="10" t="str"/>
       <x:c r="C13" s="11" t="str"/>
+      <x:c r="D13" s="25"/>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="9" t="str"/>
       <x:c r="B14" s="10" t="str"/>
       <x:c r="C14" s="11" t="str"/>
+      <x:c r="D14" s="25"/>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="9" t="str"/>
       <x:c r="B15" s="10" t="str"/>
       <x:c r="C15" s="11" t="str"/>
+      <x:c r="D15" s="25"/>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="9" t="str"/>
       <x:c r="B16" s="10" t="str"/>
       <x:c r="C16" s="11" t="str"/>
+      <x:c r="D16" s="25"/>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="9" t="str"/>
       <x:c r="B17" s="10" t="str"/>
       <x:c r="C17" s="11" t="str"/>
+      <x:c r="D17" s="25"/>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="9" t="str"/>
       <x:c r="B18" s="10" t="str"/>
       <x:c r="C18" s="11" t="str"/>
+      <x:c r="D18" s="25"/>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="9" t="str"/>
       <x:c r="B19" s="10" t="str"/>
       <x:c r="C19" s="11" t="str"/>
+      <x:c r="D19" s="25"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="9" t="str"/>
       <x:c r="B20" s="10" t="str"/>
       <x:c r="C20" s="11" t="str"/>
+      <x:c r="D20" s="25"/>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
       <x:c r="A21" s="9" t="str"/>
       <x:c r="B21" s="10" t="str"/>
       <x:c r="C21" s="11" t="str"/>
+      <x:c r="D21" s="25"/>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="9" t="str"/>
       <x:c r="B22" s="10" t="str"/>
       <x:c r="C22" s="11" t="str"/>
+      <x:c r="D22" s="25"/>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
       <x:c r="A23" s="9" t="str"/>
       <x:c r="B23" s="10" t="str"/>
       <x:c r="C23" s="11" t="str"/>
+      <x:c r="D23" s="25"/>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
       <x:c r="A24" s="9" t="str"/>
       <x:c r="B24" s="10" t="str"/>
       <x:c r="C24" s="11" t="str"/>
+      <x:c r="D24" s="25"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
       <x:c r="A25" s="9" t="str"/>
       <x:c r="B25" s="10" t="str"/>
       <x:c r="C25" s="11" t="str"/>
+      <x:c r="D25" s="25"/>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
       <x:c r="A26" s="9" t="str"/>
       <x:c r="B26" s="10" t="str"/>
       <x:c r="C26" s="11" t="str"/>
+      <x:c r="D26" s="25"/>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
       <x:c r="A27" s="9" t="str"/>
       <x:c r="B27" s="10" t="str"/>
       <x:c r="C27" s="11" t="str"/>
+      <x:c r="D27" s="25"/>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="9" t="str"/>
       <x:c r="B28" s="10" t="str"/>
       <x:c r="C28" s="11" t="str"/>
+      <x:c r="D28" s="25"/>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="9" t="str"/>
       <x:c r="B29" s="10" t="str"/>
       <x:c r="C29" s="11" t="str"/>
+      <x:c r="D29" s="25"/>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
       <x:c r="A30" s="9" t="str"/>
       <x:c r="B30" s="10" t="str"/>
       <x:c r="C30" s="11" t="str"/>
+      <x:c r="D30" s="25"/>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
       <x:c r="A31" s="9" t="str"/>
       <x:c r="B31" s="10" t="str"/>
       <x:c r="C31" s="11" t="str"/>
+      <x:c r="D31" s="25"/>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
       <x:c r="A32" s="9" t="str"/>
       <x:c r="B32" s="10" t="str"/>
       <x:c r="C32" s="11" t="str"/>
+      <x:c r="D32" s="25"/>
     </x:row>
     <x:row r="33" ht="23" customHeight="1">
       <x:c r="A33" s="9" t="str"/>
       <x:c r="B33" s="10" t="str"/>
       <x:c r="C33" s="11" t="str"/>
+      <x:c r="D33" s="25"/>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="9" t="str"/>
       <x:c r="B34" s="10" t="str"/>
       <x:c r="C34" s="11" t="str"/>
+      <x:c r="D34" s="25"/>
     </x:row>
     <x:row r="35" ht="23" customHeight="1">
       <x:c r="A35" s="9" t="str"/>
       <x:c r="B35" s="10" t="str"/>
       <x:c r="C35" s="11" t="str"/>
+      <x:c r="D35" s="25"/>
     </x:row>
     <x:row r="36" ht="23" customHeight="1">
       <x:c r="A36" s="9" t="str"/>
       <x:c r="B36" s="10" t="str"/>
       <x:c r="C36" s="11" t="str"/>
+      <x:c r="D36" s="25"/>
     </x:row>
     <x:row r="37" ht="23" customHeight="1">
       <x:c r="A37" s="9" t="str"/>
       <x:c r="B37" s="10" t="str"/>
       <x:c r="C37" s="11" t="str"/>
+      <x:c r="D37" s="25"/>
     </x:row>
     <x:row r="38" ht="23" customHeight="1">
       <x:c r="A38" s="9" t="str"/>
       <x:c r="B38" s="10" t="str"/>
       <x:c r="C38" s="11" t="str"/>
+      <x:c r="D38" s="25"/>
     </x:row>
     <x:row r="39" ht="23" customHeight="1">
       <x:c r="A39" s="9" t="str"/>
       <x:c r="B39" s="10" t="str"/>
       <x:c r="C39" s="11" t="str"/>
+      <x:c r="D39" s="25"/>
     </x:row>
     <x:row r="40" ht="23" customHeight="1">
       <x:c r="A40" s="9" t="str"/>
       <x:c r="B40" s="10" t="str"/>
       <x:c r="C40" s="11" t="str"/>
+      <x:c r="D40" s="25"/>
     </x:row>
     <x:row r="41" ht="23" customHeight="1">
       <x:c r="A41" s="9" t="str"/>
       <x:c r="B41" s="10" t="str"/>
       <x:c r="C41" s="11" t="str"/>
+      <x:c r="D41" s="25"/>
     </x:row>
     <x:row r="42" ht="23" customHeight="1">
       <x:c r="A42" s="9" t="str"/>
       <x:c r="B42" s="10" t="str"/>
       <x:c r="C42" s="11" t="str"/>
+      <x:c r="D42" s="25"/>
     </x:row>
     <x:row r="43" ht="23" customHeight="1">
       <x:c r="A43" s="9" t="str"/>
       <x:c r="B43" s="10" t="str"/>
       <x:c r="C43" s="11" t="str"/>
+      <x:c r="D43" s="25"/>
     </x:row>
     <x:row r="44" ht="23" customHeight="1">
       <x:c r="A44" s="9" t="str"/>
       <x:c r="B44" s="10" t="str"/>
       <x:c r="C44" s="11" t="str"/>
+      <x:c r="D44" s="25"/>
     </x:row>
     <x:row r="45" ht="23" customHeight="1">
       <x:c r="A45" s="9" t="str"/>
       <x:c r="B45" s="10" t="str"/>
       <x:c r="C45" s="11" t="str"/>
+      <x:c r="D45" s="25"/>
     </x:row>
     <x:row r="46" ht="23" customHeight="1">
       <x:c r="A46" s="9" t="str"/>
       <x:c r="B46" s="10" t="str"/>
       <x:c r="C46" s="11" t="str"/>
+      <x:c r="D46" s="25"/>
     </x:row>
     <x:row r="47" ht="23" customHeight="1">
       <x:c r="A47" s="9" t="str"/>
       <x:c r="B47" s="10" t="str"/>
       <x:c r="C47" s="11" t="str"/>
+      <x:c r="D47" s="25"/>
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
       <x:c r="A48" s="9" t="str"/>
       <x:c r="B48" s="10" t="str"/>
       <x:c r="C48" s="11" t="str"/>
+      <x:c r="D48" s="25"/>
     </x:row>
     <x:row r="49" ht="23" customHeight="1">
       <x:c r="A49" s="9" t="str"/>
       <x:c r="B49" s="10" t="str"/>
       <x:c r="C49" s="11" t="str"/>
+      <x:c r="D49" s="25"/>
     </x:row>
     <x:row r="50" ht="23" customHeight="1">
       <x:c r="A50" s="9" t="str"/>
       <x:c r="B50" s="10" t="str"/>
       <x:c r="C50" s="11" t="str"/>
+      <x:c r="D50" s="25"/>
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="9" t="str"/>
       <x:c r="B51" s="10" t="str"/>
       <x:c r="C51" s="11" t="str"/>
+      <x:c r="D51" s="25"/>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="D2:D51">
+      <x:formula1>"Docencia,Administrativo,LAA,PROCAME"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -678,7 +768,7 @@
         <x:v>Correo institucional con formato nombre.apellido.apellido@una.cr. No repita correos.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="34" customHeight="1">
+    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A7" s="19" t="str">
         <x:v>Contraseña temporal</x:v>
       </x:c>
@@ -686,11 +776,19 @@
         <x:v>Opcional. Déjela vacía para que el docente cree su contraseña al registrarse. Si la completa, debe tener al menos 8 caracteres, una mayúscula y un número; la cuenta se crea inmediatamente.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="34" customHeight="1">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="19" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
+        <x:v>Obligatoria. Seleccione una de estas opciones: Docencia, Administrativo, LAA o PROCAME.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A9" s="21" t="str">
         <x:v>Seguridad</x:v>
       </x:c>
-      <x:c r="B8" s="19" t="str">
+      <x:c r="B9" s="21" t="str">
         <x:v>No comparta ni conserve contraseñas innecesariamente. El profesor puede cambiarla desde su perfil.</x:v>
       </x:c>
     </x:row>

</xml_diff>